<commit_message>
daily auto-refresh 2026-09-29 15:01
</commit_message>
<xml_diff>
--- a/slab_ethnicity_matrix.xlsx
+++ b/slab_ethnicity_matrix.xlsx
@@ -673,10 +673,10 @@
         <v>104</v>
       </c>
       <c r="K6" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="L6" t="n">
-        <v>1037</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="7">
@@ -713,10 +713,10 @@
         <v>202</v>
       </c>
       <c r="K7" t="n">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="L7" t="n">
-        <v>1771</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="8">
@@ -753,10 +753,10 @@
         <v>30</v>
       </c>
       <c r="K8" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L8" t="n">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="9">
@@ -913,10 +913,10 @@
         <v>199</v>
       </c>
       <c r="K12" t="n">
-        <v>261</v>
+        <v>245</v>
       </c>
       <c r="L12" t="n">
-        <v>1100</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="13">
@@ -1912,7 +1912,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>74</v>
+        <v>67</v>
       </c>
     </row>
     <row r="48">
@@ -2712,7 +2712,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="88">
@@ -3492,7 +3492,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="127">
@@ -3812,7 +3812,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="143">
@@ -4392,7 +4392,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>177</v>
+        <v>170</v>
       </c>
     </row>
     <row r="172">
@@ -5132,7 +5132,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="209">
@@ -5852,7 +5852,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="245">
@@ -6172,7 +6172,7 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="261">
@@ -6592,7 +6592,7 @@
         </is>
       </c>
       <c r="D281" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="282">
@@ -7012,7 +7012,7 @@
         </is>
       </c>
       <c r="D302" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="303">
@@ -7232,7 +7232,7 @@
         </is>
       </c>
       <c r="D313" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="314">

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-15 15:02
</commit_message>
<xml_diff>
--- a/slab_ethnicity_matrix.xlsx
+++ b/slab_ethnicity_matrix.xlsx
@@ -553,10 +553,10 @@
         <v>59</v>
       </c>
       <c r="K3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L3" t="n">
-        <v>587</v>
+        <v>588</v>
       </c>
     </row>
     <row r="4">
@@ -593,10 +593,10 @@
         <v>69</v>
       </c>
       <c r="K4" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L4" t="n">
-        <v>713</v>
+        <v>715</v>
       </c>
     </row>
     <row r="5">
@@ -633,10 +633,10 @@
         <v>179</v>
       </c>
       <c r="K5" t="n">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="L5" t="n">
-        <v>1896</v>
+        <v>1898</v>
       </c>
     </row>
     <row r="6">
@@ -673,10 +673,10 @@
         <v>120</v>
       </c>
       <c r="K6" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="L6" t="n">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="7">
@@ -713,10 +713,10 @@
         <v>183</v>
       </c>
       <c r="K7" t="n">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="L7" t="n">
-        <v>1793</v>
+        <v>1798</v>
       </c>
     </row>
     <row r="8">
@@ -753,10 +753,10 @@
         <v>48</v>
       </c>
       <c r="K8" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="L8" t="n">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="9">
@@ -913,10 +913,10 @@
         <v>199</v>
       </c>
       <c r="K12" t="n">
-        <v>364</v>
+        <v>352</v>
       </c>
       <c r="L12" t="n">
-        <v>1220</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="13">
@@ -1952,7 +1952,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>114</v>
+        <v>104</v>
       </c>
     </row>
     <row r="50">
@@ -2352,7 +2352,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="70">
@@ -2752,7 +2752,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
     <row r="90">
@@ -2952,7 +2952,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="100">
@@ -3332,7 +3332,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="119">
@@ -3532,7 +3532,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="129">
@@ -3852,7 +3852,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="145">
@@ -4452,7 +4452,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="175">
@@ -6172,7 +6172,7 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="261">
@@ -10532,7 +10532,7 @@
         </is>
       </c>
       <c r="D478" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="479">
@@ -10972,7 +10972,7 @@
         </is>
       </c>
       <c r="D500" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="501">
@@ -11152,7 +11152,7 @@
         </is>
       </c>
       <c r="D509" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="510">

</xml_diff>